<commit_message>
De momento, estructura inicial del proyecto, cuando esté completo documento avances, esto significa que esto no está completo aún
</commit_message>
<xml_diff>
--- a/Documentacion/2. Story_Points_y_Asignacion_de_Responsabilidades.xlsx
+++ b/Documentacion/2. Story_Points_y_Asignacion_de_Responsabilidades.xlsx
@@ -744,7 +744,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="AskingMansOz" id="{9B9479FA-932F-3D27-92F8-9CB530E76C44}" userId="AskingMansOz" providerId="Teamlab"/>
+  <person displayName="AskingMansOz" id="{42AF77FE-EBC0-D0CA-E70E-7A78268B3A72}" userId="AskingMansOz" providerId="Teamlab"/>
 </personList>
 </file>
 
@@ -1203,7 +1203,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C4" dT="2026-09-23T06:07:59.81Z" personId="{9B9479FA-932F-3D27-92F8-9CB530E76C44}" id="{611E00A3-43B2-F14E-D09F-562EC24FF30B}" done="0">
+  <threadedComment ref="C4" dT="2026-09-23T06:07:59.81Z" personId="{42AF77FE-EBC0-D0CA-E70E-7A78268B3A72}" id="{611E00A3-43B2-F14E-D09F-562EC24FF30B}" done="0">
     <text xml:space="preserve">AskingMansOz:
 Mide la carga de trabajo del equipo con base en el promedio de puntos acumulados por los integrantes:
 * Verde: Por debajo del promedio (menor carga).
@@ -1253,11 +1253,11 @@
         <v>3</v>
       </c>
       <c r="C4" s="6">
-        <f>SUMIF($F$13:$F$100,B4,$E$13:$E$100)</f>
+        <f t="shared" ref="C4:C8" si="0">SUMIF($F$13:$F$100,B4,$E$13:$E$100)</f>
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>COUNTIF($F$13:$F$100,B4)</f>
+        <f t="shared" ref="D4:D8" si="1">COUNTIF($F$13:$F$100,B4)</f>
         <v>3</v>
       </c>
     </row>
@@ -1266,11 +1266,11 @@
         <v>4</v>
       </c>
       <c r="C5" s="6">
-        <f>SUMIF($F$13:$F$100,B5,$E$13:$E$100)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="D5" s="7">
-        <f>COUNTIF($F$13:$F$100,B5)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
     </row>
@@ -1279,11 +1279,11 @@
         <v>5</v>
       </c>
       <c r="C6" s="6">
-        <f>SUMIF($F$13:$F$100,B6,$E$13:$E$100)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="D6" s="7">
-        <f>COUNTIF($F$13:$F$100,B6)</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
@@ -1292,11 +1292,11 @@
         <v>6</v>
       </c>
       <c r="C7" s="6">
-        <f>SUMIF($F$13:$F$100,B7,$E$13:$E$100)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="D7" s="7">
-        <f>COUNTIF($F$13:$F$100,B7)</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
     </row>
@@ -1305,11 +1305,11 @@
         <v>7</v>
       </c>
       <c r="C8" s="6">
-        <f>SUMIF($F$13:$F$100,B8,$E$13:$E$100)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="D8" s="10">
-        <f>COUNTIF($F$13:$F$100,B8)</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="H8" s="11"/>
@@ -1598,6 +1598,7 @@
     <row r="34" ht="57" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="8BS5AFDeWUp2uXkKLLl8ly842sWzr9SnZl7yXA4vXP6V9XfoW3pgR5z7lHslR5YkWRDBTAO47cvP/wC6qeaHrg==" saltValue="ip0g8D5p8msBvm9OXhJ/Qw==" spinCount="100000" autoFilter="1" deleteColumns="1" deleteRows="1" formatCells="1" formatColumns="1" formatRows="1" insertColumns="1" insertHyperlinks="1" insertRows="1" objects="1" pivotTables="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1" sheet="1" sort="1"/>
   <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.51181102362204689" footer="0.51181102362204689"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1607,7 +1608,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="aboveAverage" priority="6" stdDev="0" id="{A98D0DC9-7E84-49A3-9310-86BF2E756876}">
+          <x14:cfRule type="aboveAverage" priority="6" stdDev="0" id="{2D8B64D1-FB8F-4B6B-84E0-F677FA877FB3}">
             <x14:dxf>
               <font>
                 <color rgb="FF9C0006"/>
@@ -1623,7 +1624,7 @@
           <xm:sqref>C4:C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="aboveAverage" priority="5" stdDev="0" id="{DC113D19-2C5B-4826-9E2C-C6B88FA63ADD}">
+          <x14:cfRule type="aboveAverage" priority="5" stdDev="0" id="{9240CF11-6FB7-4565-B702-7638449FBFD3}">
             <x14:dxf>
               <font>
                 <color rgb="FF9C0006"/>
@@ -1639,7 +1640,7 @@
           <xm:sqref>C4:C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="aboveAverage" priority="4" aboveAverage="0" stdDev="0" id="{264F6DCF-4F82-4CFF-A418-837729AFDCB6}">
+          <x14:cfRule type="aboveAverage" priority="4" aboveAverage="0" stdDev="0" id="{C8034D67-DE06-485D-A56C-04ED30333175}">
             <x14:dxf>
               <font>
                 <color rgb="FF006100"/>
@@ -1655,7 +1656,7 @@
           <xm:sqref>C4:C8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="3" operator="greaterThan" id="{55D81D1C-5D79-4BBA-AA6B-BA5BECCBB855}">
+          <x14:cfRule type="cellIs" priority="3" operator="greaterThan" id="{175B8E6F-B499-4ED5-B87B-DB230E9AB56C}">
             <xm:f>5</xm:f>
             <x14:dxf>
               <font>
@@ -1672,7 +1673,7 @@
           <xm:sqref>E13:E26</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="lessThan" id="{6F5C3A98-FABA-4F0B-B895-C81830766983}">
+          <x14:cfRule type="cellIs" priority="2" operator="lessThan" id="{85DA5DD3-6291-4E46-B442-6962E391F98C}">
             <xm:f>5</xm:f>
             <x14:dxf>
               <font>
@@ -1689,7 +1690,7 @@
           <xm:sqref>E13:E26</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{B609CB1D-724C-4396-B1F1-00F3D1D72AFF}">
+          <x14:cfRule type="cellIs" priority="1" operator="equal" id="{2D39660B-5339-4C74-AF9E-19FA65971520}">
             <xm:f>5</xm:f>
             <x14:dxf>
               <font>
@@ -1709,7 +1710,7 @@
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2" disablePrompts="0">
-        <x14:dataValidation xr:uid="{CE911A5F-022B-4DE6-B346-615E7E7FEEEC}" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{13F79E6A-81B2-4ECD-8322-0994804E9EDE}" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>0</xm:f>
           </x14:formula1>
@@ -1718,7 +1719,7 @@
           </x14:formula2>
           <xm:sqref>B4:B8</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{28373C1C-3FBA-498C-B488-E9429F39B879}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{4CBF71D5-E3D2-4EB7-A748-2244BF99187A}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$B$4:$B$8</xm:f>
           </x14:formula1>

</xml_diff>